<commit_message>
feat: a sheet can name one colour for the whole card
`#config theme=sakura` paints the card in a named palette instead of leaving it
black on white. A theme also redefines what `color=muted` and `color=accent`
mean, so a column styled with either follows the sheet's palette rather than
staying the same blue on every card.

Each palette carries a light and a dark half, because Anki decides at review
time which one a card is drawn in — one set of colours would leave the other
mode unreadable. The card is painted through `.card` / `.card.night_mode`: two
classes, so the rule outranks the single-class night-mode rule Anki's own
stylesheet brings. Without a theme nothing paints the card at all, so an
untouched sheet keeps the colours it had.

An unknown name is refused by name in the warnings and the card keeps Anki's
colours. The preview's iframe now carries `night_mode` alongside `card`, as
Anki does, or a dark page would show the light half of the theme.
</commit_message>
<xml_diff>
--- a/examples/sheets2anki-examples.xlsx
+++ b/examples/sheets2anki-examples.xlsx
@@ -2581,7 +2581,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">#config align=left; speed=0.9; reverse</t>
+          <t xml:space="preserve">#config align=left; speed=0.9; reverse; theme=sakura</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -3116,7 +3116,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">#config align=middle; spid=3; reverse</t>
+          <t xml:space="preserve">#config align=middle; spid=3; reverse; theme=neon</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">

</xml_diff>

<commit_message>
feat: a sheet can name the deck for the rows that name none
A row with every SUBDECK cell empty was never unfiled — Anki has no such
state — but it landed in the sheet's own deck, mixed in with the rows that
were filed. `#config unsorted=Chưa phân loại` gives those rows a deck of
their own; the bare flag calls it `Unsorted`.

Nothing is invented: without the key a sheet behaves exactly as before,
because a name the add-on chose would arrive in English in a deck list that
is not. It is applied in `deck_path` as the single level of an otherwise
empty path, so the deck and the mirrored tag follow from one place, and a
partly-filled path is left alone.
</commit_message>
<xml_diff>
--- a/examples/sheets2anki-examples.xlsx
+++ b/examples/sheets2anki-examples.xlsx
@@ -3116,7 +3116,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">#config align=middle; spid=3; reverse; theme=neon</t>
+          <t xml:space="preserve">#config align=middle; spid=3; reverse; theme=neon; unsorted=</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -3352,49 +3352,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">s01</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Geography</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Capitals</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">europe, capitals</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Capital of Portugal?</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lisbon</t>
+          <t xml:space="preserve">#config unsorted=Unsorted</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">s02</t>
+          <t xml:space="preserve">s01</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">x</t>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3409,29 +3379,29 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">asia; capitals</t>
+          <t xml:space="preserve">europe, capitals</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Capital of Vietnam?</t>
+          <t xml:space="preserve">Capital of Portugal?</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hanoi</t>
+          <t xml:space="preserve">Lisbon</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">s03</t>
+          <t xml:space="preserve">s02</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">x</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -3441,34 +3411,34 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rivers</t>
+          <t xml:space="preserve">Capitals</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">rivers</t>
+          <t xml:space="preserve">asia; capitals</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Longest river in Asia?</t>
+          <t xml:space="preserve">Capital of Vietnam?</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Yangtze</t>
+          <t xml:space="preserve">Hanoi</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">s04</t>
+          <t xml:space="preserve">s03</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRUE</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -3483,133 +3453,170 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">rivers, europe</t>
+          <t xml:space="preserve">rivers</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Which river flows through Paris?</t>
+          <t xml:space="preserve">Longest river in Asia?</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Seine</t>
+          <t xml:space="preserve">The Yangtze</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">s05</t>
+          <t xml:space="preserve">s04</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">✓</t>
+          <t xml:space="preserve">TRUE</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">History</t>
+          <t xml:space="preserve">Geography</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rivers</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">history</t>
+          <t xml:space="preserve">rivers, europe</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Who was the first Ming emperor?</t>
+          <t xml:space="preserve">Which river flows through Paris?</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Hongwu Emperor</t>
+          <t xml:space="preserve">The Seine</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">s06</t>
+          <t xml:space="preserve">s05</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">✓</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">History</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">history</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve">A row with no SUBDECK stays in the deck root.</t>
+          <t xml:space="preserve">Who was the first Ming emperor?</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t xml:space="preserve">No subdeck, no tag.</t>
+          <t xml:space="preserve">The Hongwu Emperor</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">s07</t>
+          <t xml:space="preserve">s06</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">no</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Geography</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Capitals</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">capitals</t>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve">This row is switched off.</t>
+          <t xml:space="preserve">Where does a row with both SUBDECK cells empty go?</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t xml:space="preserve">It is never written to Anki.</t>
+          <t xml:space="preserve">Into 'Unsorted', because the settings row named it. Without that key it stays in the sheet's own deck, beside the sub-decks.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t xml:space="preserve">s07</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Geography</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Capitals</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">capitals</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This row is switched off.</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">It is never written to Anki.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t xml:space="preserve">s08</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t xml:space="preserve">History</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t xml:space="preserve">history</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t xml:space="preserve">An empty SYNC cell is off too.</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t xml:space="preserve">Same as 'no'.</t>
         </is>

</xml_diff>

<commit_message>
feat: the unsorted pile is automatic, and the directive is gone
`#config unsorted=<name>` lasted one version. A sheet that sorts its rows into
sub-decks is already saying that a row belongs somewhere, so the row that names
no level has an answer either way — and the key could only ever have been a way
to ask for those rows to stay loose among the folders.

So it happens by itself: a row with no level lands in `Unsorted`, named in
English because that is the word every spreadsheet already uses for the pile.
Applied in `deck_path` as the single level of an otherwise empty path, so the
deck and the mirrored tag follow from one place.

It fires only on a sheet that has levels at all. With nothing to be unsorted
from, a two-column vocabulary sheet would otherwise find every one of its notes
moved into a folder — which is a level of deck nobody asked for.

The blank-SUBDECK tag changes with it: `sheets2anki::unsorted` instead of no tag
at all. It mirrors the deck, as every deck tag does.
</commit_message>
<xml_diff>
--- a/examples/sheets2anki-examples.xlsx
+++ b/examples/sheets2anki-examples.xlsx
@@ -3116,7 +3116,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">#config align=middle; spid=3; reverse; theme=neon; unsorted=</t>
+          <t xml:space="preserve">#config align=middle; spid=3; reverse; theme=neon</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -3352,19 +3352,49 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">#config unsorted=Unsorted</t>
+          <t xml:space="preserve">s01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Geography</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Capitals</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">europe, capitals</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Capital of Portugal?</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lisbon</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">s01</t>
+          <t xml:space="preserve">s02</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">x</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3379,29 +3409,29 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">europe, capitals</t>
+          <t xml:space="preserve">asia; capitals</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Capital of Portugal?</t>
+          <t xml:space="preserve">Capital of Vietnam?</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lisbon</t>
+          <t xml:space="preserve">Hanoi</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">s02</t>
+          <t xml:space="preserve">s03</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">x</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -3411,34 +3441,34 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Capitals</t>
+          <t xml:space="preserve">Rivers</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">asia; capitals</t>
+          <t xml:space="preserve">rivers</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Capital of Vietnam?</t>
+          <t xml:space="preserve">Longest river in Asia?</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hanoi</t>
+          <t xml:space="preserve">The Yangtze</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">s03</t>
+          <t xml:space="preserve">s04</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">TRUE</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -3453,170 +3483,133 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">rivers</t>
+          <t xml:space="preserve">rivers, europe</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Longest river in Asia?</t>
+          <t xml:space="preserve">Which river flows through Paris?</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Yangtze</t>
+          <t xml:space="preserve">The Seine</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">s04</t>
+          <t xml:space="preserve">s05</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRUE</t>
+          <t xml:space="preserve">✓</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Geography</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Rivers</t>
+          <t xml:space="preserve">History</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">rivers, europe</t>
+          <t xml:space="preserve">history</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Which river flows through Paris?</t>
+          <t xml:space="preserve">Who was the first Ming emperor?</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Seine</t>
+          <t xml:space="preserve">The Hongwu Emperor</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">s05</t>
+          <t xml:space="preserve">s06</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">✓</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">History</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">history</t>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Who was the first Ming emperor?</t>
+          <t xml:space="preserve">Where does a row with both SUBDECK cells empty go?</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Hongwu Emperor</t>
+          <t xml:space="preserve">Into 'Unsorted'. A sheet that sorts its rows has somewhere for the ones it did not sort.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">s06</t>
+          <t xml:space="preserve">s07</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">no</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Geography</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Capitals</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">capitals</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Where does a row with both SUBDECK cells empty go?</t>
+          <t xml:space="preserve">This row is switched off.</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Into 'Unsorted', because the settings row named it. Without that key it stays in the sheet's own deck, beside the sub-decks.</t>
+          <t xml:space="preserve">It is never written to Anki.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">s07</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">no</t>
+          <t xml:space="preserve">s08</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Geography</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Capitals</t>
+          <t xml:space="preserve">History</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">capitals</t>
+          <t xml:space="preserve">history</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t xml:space="preserve">This row is switched off.</t>
+          <t xml:space="preserve">An empty SYNC cell is off too.</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">It is never written to Anki.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">s08</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">History</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">history</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">An empty SYNC cell is off too.</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
         <is>
           <t xml:space="preserve">Same as 'no'.</t>
         </is>

</xml_diff>

<commit_message>
refactor: the sheet the site opens on is English
Sheet 15 is the first thing anyone sees: it is the widest sheet, so it is the one
the preview page opens on, and it was a JLPT list in Japanese. Someone arriving to
find out what this add-on does should not have to read a script they do not know
before they can tell what they are looking at.

Same directives, same shape, English words: `English::B1::Verbs` three levels
deep, `theme=sakura` over the whole card, the word spoken and the example spoken
slower, tagged by CEFR level, and `sort` so the browser lists the words instead of
n01, n02, n03. `furigana` goes with the Japanese — sheet 13 is where it belongs
and where it stays.
</commit_message>
<xml_diff>
--- a/examples/sheets2anki-examples.xlsx
+++ b/examples/sheets2anki-examples.xlsx
@@ -2549,15 +2549,20 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Japanese</t>
+          <t xml:space="preserve">Word</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t xml:space="preserve">Phonetic</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Meaning</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t xml:space="preserve">Example</t>
         </is>
@@ -2571,17 +2576,22 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve">size=40; furigana; tts=ja_JP</t>
+          <t xml:space="preserve">size=44; bold; tts=en_US; sort</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t xml:space="preserve">side=back; size=20; color=accent</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t xml:space="preserve">side=back; size=22</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">side=back; size=16; color=muted; italic; furigana</t>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">side=back; size=16; color=muted; italic; tts=en_US; speed=0.85</t>
         </is>
       </c>
     </row>
@@ -2593,12 +2603,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">JLPT</t>
+          <t xml:space="preserve">English</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">N5</t>
+          <t xml:space="preserve">B1</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -2608,22 +2618,27 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">jlpt, n5</t>
+          <t xml:space="preserve">cefr, b1</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve">食[た]べる</t>
+          <t xml:space="preserve">to afford</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ăn</t>
+          <t xml:space="preserve">/əˈfɔːd/</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t xml:space="preserve">朝[あさ]ごはんを 食[た]べます。</t>
+          <t xml:space="preserve">đủ tiền để mua</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">We cannot afford a bigger flat this year.</t>
         </is>
       </c>
     </row>
@@ -2635,12 +2650,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">JLPT</t>
+          <t xml:space="preserve">English</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">N5</t>
+          <t xml:space="preserve">B1</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -2650,22 +2665,27 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">jlpt, n5</t>
+          <t xml:space="preserve">cefr, b1</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve">飲[の]む</t>
+          <t xml:space="preserve">to complain</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t xml:space="preserve">uống</t>
+          <t xml:space="preserve">/kəmˈpleɪn/</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t xml:space="preserve">毎朝[まいあさ] コーヒーを 飲[の]みます。</t>
+          <t xml:space="preserve">phàn nàn</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">She complained about the noise upstairs.</t>
         </is>
       </c>
     </row>
@@ -2677,12 +2697,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">JLPT</t>
+          <t xml:space="preserve">English</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">N5</t>
+          <t xml:space="preserve">B1</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -2692,22 +2712,27 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">jlpt, n5</t>
+          <t xml:space="preserve">cefr, b1</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve">行[い]く</t>
+          <t xml:space="preserve">to improve</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t xml:space="preserve">đi</t>
+          <t xml:space="preserve">/ɪmˈpruːv/</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t xml:space="preserve">来週[らいしゅう] 京都[きょうと]へ 行[い]きます。</t>
+          <t xml:space="preserve">cải thiện</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">His English improved after a year in Leeds.</t>
         </is>
       </c>
     </row>
@@ -2719,12 +2744,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">JLPT</t>
+          <t xml:space="preserve">English</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">N5</t>
+          <t xml:space="preserve">B1</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -2734,22 +2759,27 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">jlpt, n5</t>
+          <t xml:space="preserve">cefr, b1</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve">話[はな]す</t>
+          <t xml:space="preserve">to suggest</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t xml:space="preserve">nói chuyện</t>
+          <t xml:space="preserve">/səˈdʒest/</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t xml:space="preserve">日本語[にほんご]で 話[はな]しましょう。</t>
+          <t xml:space="preserve">gợi ý, đề nghị</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I suggest leaving before the traffic starts.</t>
         </is>
       </c>
     </row>
@@ -2761,12 +2791,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">JLPT</t>
+          <t xml:space="preserve">English</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">N5</t>
+          <t xml:space="preserve">B1</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -2776,22 +2806,27 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">jlpt, n5</t>
+          <t xml:space="preserve">cefr, b1</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve">学校[がっこう]</t>
+          <t xml:space="preserve">advice</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t xml:space="preserve">trường học</t>
+          <t xml:space="preserve">/ədˈvaɪs/</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t xml:space="preserve">学校[がっこう]は 駅[えき]の 近[ちか]くです。</t>
+          <t xml:space="preserve">lời khuyên</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">She gave me some good advice.</t>
         </is>
       </c>
     </row>
@@ -2803,12 +2838,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">JLPT</t>
+          <t xml:space="preserve">English</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">N5</t>
+          <t xml:space="preserve">B1</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -2818,22 +2853,27 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">jlpt, n5</t>
+          <t xml:space="preserve">cefr, b1</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve">友[とも]だち</t>
+          <t xml:space="preserve">journey</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t xml:space="preserve">bạn bè</t>
+          <t xml:space="preserve">/ˈdʒɜːni/</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t xml:space="preserve">友[とも]だちと 映画[えいが]を 見[み]ました。</t>
+          <t xml:space="preserve">chuyến đi</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The journey takes about four hours.</t>
         </is>
       </c>
     </row>
@@ -2845,12 +2885,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">JLPT</t>
+          <t xml:space="preserve">English</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">N5</t>
+          <t xml:space="preserve">B1</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -2860,22 +2900,27 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t xml:space="preserve">jlpt, n5</t>
+          <t xml:space="preserve">cefr, b1</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t xml:space="preserve">電車[でんしゃ]</t>
+          <t xml:space="preserve">neighbour</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t xml:space="preserve">tàu điện</t>
+          <t xml:space="preserve">/ˈneɪbə/</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t xml:space="preserve">電車[でんしゃ]で 会社[かいしゃ]へ 行[い]きます。</t>
+          <t xml:space="preserve">hàng xóm</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Our neighbour looks after the cat.</t>
         </is>
       </c>
     </row>
@@ -2887,37 +2932,42 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">JLPT</t>
+          <t xml:space="preserve">English</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">N5</t>
+          <t xml:space="preserve">B1</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nouns</t>
+          <t xml:space="preserve">Adjectives</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">jlpt, n5</t>
+          <t xml:space="preserve">cefr, b1</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t xml:space="preserve">時間[じかん]</t>
+          <t xml:space="preserve">crowded</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t xml:space="preserve">thời gian</t>
+          <t xml:space="preserve">/ˈkraʊdɪd/</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t xml:space="preserve">今日[きょう]は 時間[じかん]が ありません。</t>
+          <t xml:space="preserve">đông đúc</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The market is crowded on Sunday mornings.</t>
         </is>
       </c>
     </row>
@@ -2929,12 +2979,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">JLPT</t>
+          <t xml:space="preserve">English</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">N5</t>
+          <t xml:space="preserve">B1</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -2944,22 +2994,27 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">jlpt, n5</t>
+          <t xml:space="preserve">cefr, b1</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve">新[あたら]しい</t>
+          <t xml:space="preserve">reliable</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t xml:space="preserve">mới</t>
+          <t xml:space="preserve">/rɪˈlaɪəbl/</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t xml:space="preserve">新[あたら]しい 本[ほん]を 買[か]いました。</t>
+          <t xml:space="preserve">đáng tin cậy</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">He is the most reliable person on the team.</t>
         </is>
       </c>
     </row>
@@ -2971,37 +3026,42 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">JLPT</t>
+          <t xml:space="preserve">English</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">N5</t>
+          <t xml:space="preserve">B2</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Adjectives</t>
+          <t xml:space="preserve">Verbs</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">jlpt, n5</t>
+          <t xml:space="preserve">cefr, b2</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t xml:space="preserve">高[たか]い</t>
+          <t xml:space="preserve">to acknowledge</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t xml:space="preserve">cao; đắt</t>
+          <t xml:space="preserve">/əkˈnɒlɪdʒ/</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t xml:space="preserve">この 店[みせ]は 少[すこ]し 高[たか]いです。</t>
+          <t xml:space="preserve">thừa nhận</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">She acknowledged that the plan had failed.</t>
         </is>
       </c>
     </row>
@@ -3013,37 +3073,42 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">JLPT</t>
+          <t xml:space="preserve">English</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">N5</t>
+          <t xml:space="preserve">B2</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Adjectives</t>
+          <t xml:space="preserve">Verbs</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">jlpt, n5</t>
+          <t xml:space="preserve">cefr, b2</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t xml:space="preserve">静[しず]か</t>
+          <t xml:space="preserve">to postpone</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t xml:space="preserve">yên tĩnh</t>
+          <t xml:space="preserve">/pəˈspəʊn/</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t xml:space="preserve">この 部屋[へや]は とても 静[しず]かです。</t>
+          <t xml:space="preserve">hoãn lại</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">They postponed the concert until March.</t>
         </is>
       </c>
     </row>
@@ -3055,37 +3120,42 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">JLPT</t>
+          <t xml:space="preserve">English</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">N4</t>
+          <t xml:space="preserve">B2</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Verbs</t>
+          <t xml:space="preserve">Nouns</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t xml:space="preserve">jlpt, n4</t>
+          <t xml:space="preserve">cefr, b2</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t xml:space="preserve">調[しら]べる</t>
+          <t xml:space="preserve">assumption</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t xml:space="preserve">tra cứu; tìm hiểu</t>
+          <t xml:space="preserve">/əˈsʌmpʃn/</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t xml:space="preserve">辞書[じしょ]で 言葉[ことば]を 調[しら]べます。</t>
+          <t xml:space="preserve">giả định</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The whole plan rests on one assumption.</t>
         </is>
       </c>
     </row>
@@ -3097,37 +3167,42 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">JLPT</t>
+          <t xml:space="preserve">English</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">N4</t>
+          <t xml:space="preserve">B2</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Verbs</t>
+          <t xml:space="preserve">Nouns</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">jlpt, n4</t>
+          <t xml:space="preserve">cefr, b2</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t xml:space="preserve">続[つづ]ける</t>
+          <t xml:space="preserve">consequence</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t xml:space="preserve">tiếp tục</t>
+          <t xml:space="preserve">/ˈkɒnsɪkwəns/</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t xml:space="preserve">毎日[まいにち] 練習[れんしゅう]を 続[つづ]けます。</t>
+          <t xml:space="preserve">hậu quả</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nobody thought about the consequences.</t>
         </is>
       </c>
     </row>
@@ -3139,37 +3214,42 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">JLPT</t>
+          <t xml:space="preserve">English</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">N4</t>
+          <t xml:space="preserve">B2</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nouns</t>
+          <t xml:space="preserve">Adjectives</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t xml:space="preserve">jlpt, n4</t>
+          <t xml:space="preserve">cefr, b2</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t xml:space="preserve">季節[きせつ]</t>
+          <t xml:space="preserve">thorough</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t xml:space="preserve">mùa</t>
+          <t xml:space="preserve">/ˈθʌrə/</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t xml:space="preserve">日本[にほん]には 四[よっ]つの 季節[きせつ]が あります。</t>
+          <t xml:space="preserve">kỹ lưỡng</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The report was thorough and easy to read.</t>
         </is>
       </c>
     </row>
@@ -3181,37 +3261,42 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">JLPT</t>
+          <t xml:space="preserve">English</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">N4</t>
+          <t xml:space="preserve">B2</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nouns</t>
+          <t xml:space="preserve">Adjectives</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t xml:space="preserve">jlpt, n4</t>
+          <t xml:space="preserve">cefr, b2</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t xml:space="preserve">桜[さくら]</t>
+          <t xml:space="preserve">reluctant</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t xml:space="preserve">hoa anh đào</t>
+          <t xml:space="preserve">/rɪˈlʌktənt/</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t xml:space="preserve">春[はる]に 桜[さくら]が 咲[さ]きます。</t>
+          <t xml:space="preserve">miễn cưỡng</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">He was reluctant to answer the question.</t>
         </is>
       </c>
     </row>

</xml_diff>